<commit_message>
Premarca títulos obvios en la validación y corrige casos detectados en la muestra
- La planilla marca «si» los títulos que nombran la dirección o gestión escolar
  (editable); quedan 144 de 200 para revisar a mano.
- Una mención a covid, salud o ESI ya no descarta un trabajo que relaciona
  gestión y escuela.
- «community management» como tipo de sostenimiento.
- Se excluyen las guías de biblioteca (LibGuides), que no son trabajos académicos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YizmwDcS699vYHXm3rbDZ
</commit_message>
<xml_diff>
--- a/data/validacion/muestra_pertinencia.xlsx
+++ b/data/validacion/muestra_pertinencia.xlsx
@@ -12,7 +12,9 @@
     <sheet name="Estratos" sheetId="3" state="hidden" r:id="rId3"/>
     <sheet name="Poblacion" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Muestra'!$A$1:$L$201</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -434,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -447,9 +449,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -474,12 +474,26 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>La planilla no muestra qué decidió el filtro, para no condicionar la lectura.</t>
+          <t>Los títulos que nombran explícitamente la dirección o gestión escolar ya vienen marcados «si» (columna «marcado_por»); se pueden corregir.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>Para ver solo lo pendiente: filtro del encabezado «pertinente» → (Vacías).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>La planilla no muestra qué decidió el filtro, para no condicionar la lectura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Al terminar: python scripts/evaluate_relevance_validation.py</t>
         </is>
@@ -496,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K201"/>
+  <dimension ref="A1:L201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -563,7 +577,12 @@
           <t>pertinente</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>marcado_por</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>nota</t>
         </is>
@@ -606,7 +625,7 @@
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -652,8 +671,17 @@
           <t>https://doi.org/10.5281/zenodo.17518914</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -692,7 +720,7 @@
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -735,7 +763,7 @@
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -777,8 +805,17 @@
           <t>https://research.monash.edu/en/publications/exploring-intersections-of-educational-leadership-educational-cha</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -824,8 +861,17 @@
           <t>https://doi.org/10.5281/zenodo.6966871</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -872,7 +918,7 @@
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -919,7 +965,7 @@
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -966,7 +1012,7 @@
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1009,7 +1055,7 @@
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1048,7 +1094,7 @@
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1094,8 +1140,8 @@
           <t>https://guides.lib.uni.edu/school-management</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="n"/>
+      <c r="L13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1134,7 +1180,7 @@
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1180,8 +1226,17 @@
           <t>https://doi.org/10.31619/caledu.n56.1189</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1223,7 +1278,7 @@
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1262,7 +1317,7 @@
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1304,8 +1359,17 @@
           <t>https://doi.org/10.1007/978-3-030-39666-4_120-1</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1344,7 +1408,7 @@
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1391,7 +1455,7 @@
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1430,7 +1494,7 @@
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1477,7 +1541,7 @@
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr"/>
-      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1516,7 +1580,7 @@
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1562,8 +1626,17 @@
           <t>https://doi.org/10.1177/17411432211019407</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1602,7 +1675,7 @@
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1642,7 +1715,7 @@
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1681,7 +1754,7 @@
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1728,7 +1801,7 @@
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1775,7 +1848,7 @@
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1818,7 +1891,7 @@
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -1857,7 +1930,7 @@
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -1904,7 +1977,7 @@
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -1943,7 +2016,7 @@
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -1982,7 +2055,7 @@
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2024,8 +2097,17 @@
           <t>https://doi.org/10.1257/rct.17236-1.1</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2071,8 +2153,17 @@
           <t>https://doi.org/10.59231/sari7600</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2119,7 +2210,7 @@
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr"/>
-      <c r="K37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2158,7 +2249,7 @@
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
+      <c r="L38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2197,7 +2288,7 @@
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr"/>
-      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -2244,7 +2335,7 @@
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr"/>
+      <c r="L40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -2291,7 +2382,7 @@
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr"/>
-      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -2338,7 +2429,7 @@
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr"/>
-      <c r="K42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -2384,8 +2475,17 @@
           <t>http://dx.doi.org/10.26820/recimundo/8.(2).abril.2024.406-421</t>
         </is>
       </c>
-      <c r="J43" s="3" t="inlineStr"/>
-      <c r="K43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2424,7 +2524,7 @@
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr"/>
-      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -2471,7 +2571,7 @@
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr"/>
-      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -2510,7 +2610,7 @@
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr"/>
-      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -2549,7 +2649,7 @@
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr"/>
-      <c r="K47" s="3" t="inlineStr"/>
+      <c r="L47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -2591,8 +2691,17 @@
           <t>https://doi.org/10.5040/9798881830403.ch-010</t>
         </is>
       </c>
-      <c r="J48" s="3" t="inlineStr"/>
-      <c r="K48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -2638,8 +2747,17 @@
           <t>https://doi.org/10.46932/sfjdv2n2-062</t>
         </is>
       </c>
-      <c r="J49" s="3" t="inlineStr"/>
-      <c r="K49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -2686,7 +2804,7 @@
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr"/>
-      <c r="K50" s="3" t="inlineStr"/>
+      <c r="L50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -2733,7 +2851,7 @@
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr"/>
-      <c r="K51" s="3" t="inlineStr"/>
+      <c r="L51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -2772,7 +2890,7 @@
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr"/>
-      <c r="K52" s="3" t="inlineStr"/>
+      <c r="L52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -2819,7 +2937,7 @@
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr"/>
-      <c r="K53" s="3" t="inlineStr"/>
+      <c r="L53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -2858,7 +2976,7 @@
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr"/>
-      <c r="K54" s="3" t="inlineStr"/>
+      <c r="L54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -2897,7 +3015,7 @@
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr"/>
-      <c r="K55" s="3" t="inlineStr"/>
+      <c r="L55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -2944,7 +3062,7 @@
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr"/>
-      <c r="K56" s="3" t="inlineStr"/>
+      <c r="L56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -2983,7 +3101,7 @@
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr"/>
-      <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -3022,7 +3140,7 @@
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr"/>
-      <c r="K58" s="3" t="inlineStr"/>
+      <c r="L58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -3068,8 +3186,17 @@
           <t>https://doi.org/10.20944/preprints202206.0418.v1</t>
         </is>
       </c>
-      <c r="J59" s="3" t="inlineStr"/>
-      <c r="K59" s="3" t="inlineStr"/>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -3108,7 +3235,7 @@
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr"/>
-      <c r="K60" s="3" t="inlineStr"/>
+      <c r="L60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -3154,8 +3281,17 @@
           <t>https://doi.org/10.61728/ae24080088</t>
         </is>
       </c>
-      <c r="J61" s="3" t="inlineStr"/>
-      <c r="K61" s="3" t="inlineStr"/>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -3202,7 +3338,7 @@
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr"/>
-      <c r="K62" s="3" t="inlineStr"/>
+      <c r="L62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -3241,7 +3377,7 @@
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr"/>
-      <c r="K63" s="3" t="inlineStr"/>
+      <c r="L63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -3288,7 +3424,7 @@
         </is>
       </c>
       <c r="J64" s="3" t="inlineStr"/>
-      <c r="K64" s="3" t="inlineStr"/>
+      <c r="L64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -3335,7 +3471,7 @@
         </is>
       </c>
       <c r="J65" s="3" t="inlineStr"/>
-      <c r="K65" s="3" t="inlineStr"/>
+      <c r="L65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -3374,7 +3510,7 @@
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr"/>
-      <c r="K66" s="3" t="inlineStr"/>
+      <c r="L66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -3413,7 +3549,7 @@
         </is>
       </c>
       <c r="J67" s="3" t="inlineStr"/>
-      <c r="K67" s="3" t="inlineStr"/>
+      <c r="L67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -3455,8 +3591,17 @@
           <t>https://doi.org/10.1007/978-3-032-21359-4_194</t>
         </is>
       </c>
-      <c r="J68" s="3" t="inlineStr"/>
-      <c r="K68" s="3" t="inlineStr"/>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -3495,7 +3640,7 @@
         </is>
       </c>
       <c r="J69" s="3" t="inlineStr"/>
-      <c r="K69" s="3" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -3534,7 +3679,7 @@
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr"/>
-      <c r="K70" s="3" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -3572,8 +3717,17 @@
           <t>http://hdl.handle.net/11336/124038</t>
         </is>
       </c>
-      <c r="J71" s="3" t="inlineStr"/>
-      <c r="K71" s="3" t="inlineStr"/>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -3619,8 +3773,17 @@
           <t>http://dx.doi.org/10.4324/9781003279334-9</t>
         </is>
       </c>
-      <c r="J72" s="3" t="inlineStr"/>
-      <c r="K72" s="3" t="inlineStr"/>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -3667,7 +3830,7 @@
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr"/>
-      <c r="K73" s="3" t="inlineStr"/>
+      <c r="L73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -3706,7 +3869,7 @@
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr"/>
-      <c r="K74" s="3" t="inlineStr"/>
+      <c r="L74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -3745,7 +3908,7 @@
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr"/>
-      <c r="K75" s="3" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -3784,7 +3947,7 @@
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr"/>
-      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -3831,7 +3994,7 @@
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr"/>
-      <c r="K77" s="3" t="inlineStr"/>
+      <c r="L77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -3870,7 +4033,7 @@
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr"/>
-      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -3909,7 +4072,7 @@
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr"/>
-      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -3955,8 +4118,17 @@
           <t>https://app.trdizin.gov.tr/makale/TkRJNU1qSTRPQT09/being-a-woman-school-principal-in-turkey</t>
         </is>
       </c>
-      <c r="J80" s="3" t="inlineStr"/>
-      <c r="K80" s="3" t="inlineStr"/>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -3998,8 +4170,17 @@
           <t>https://doi.org/10.5040/9781350160552.0009</t>
         </is>
       </c>
-      <c r="J81" s="3" t="inlineStr"/>
-      <c r="K81" s="3" t="inlineStr"/>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -4038,7 +4219,7 @@
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr"/>
-      <c r="K82" s="3" t="inlineStr"/>
+      <c r="L82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -4084,8 +4265,17 @@
           <t>https://doi.org/10.71068/ybw06p77</t>
         </is>
       </c>
-      <c r="J83" s="3" t="inlineStr"/>
-      <c r="K83" s="3" t="inlineStr"/>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -4132,7 +4322,7 @@
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr"/>
-      <c r="K84" s="3" t="inlineStr"/>
+      <c r="L84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -4171,7 +4361,7 @@
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr"/>
-      <c r="K85" s="3" t="inlineStr"/>
+      <c r="L85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -4218,7 +4408,7 @@
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr"/>
-      <c r="K86" s="3" t="inlineStr"/>
+      <c r="L86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -4265,7 +4455,7 @@
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr"/>
-      <c r="K87" s="3" t="inlineStr"/>
+      <c r="L87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -4306,7 +4496,7 @@
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr"/>
-      <c r="K88" s="3" t="inlineStr"/>
+      <c r="L88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -4344,8 +4534,17 @@
           <t>http://hdl.handle.net/11336/297986</t>
         </is>
       </c>
-      <c r="J89" s="3" t="inlineStr"/>
-      <c r="K89" s="3" t="inlineStr"/>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -4384,7 +4583,7 @@
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr"/>
-      <c r="K90" s="3" t="inlineStr"/>
+      <c r="L90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n">
@@ -4430,8 +4629,17 @@
           <t>http://dx.doi.org/10.17583/ijelm.12766</t>
         </is>
       </c>
-      <c r="J91" s="3" t="inlineStr"/>
-      <c r="K91" s="3" t="inlineStr"/>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n">
@@ -4477,8 +4685,17 @@
           <t>https://doi.org/10.29228/sobider.65006</t>
         </is>
       </c>
-      <c r="J92" s="3" t="inlineStr"/>
-      <c r="K92" s="3" t="inlineStr"/>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
@@ -4516,8 +4733,17 @@
           <t>http://hdl.handle.net/11336/126296</t>
         </is>
       </c>
-      <c r="J93" s="3" t="inlineStr"/>
-      <c r="K93" s="3" t="inlineStr"/>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L93" s="3" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -4564,7 +4790,7 @@
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr"/>
-      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -4602,8 +4828,17 @@
           <t>http://hdl.handle.net/11336/228877</t>
         </is>
       </c>
-      <c r="J95" s="3" t="inlineStr"/>
-      <c r="K95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L95" s="3" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -4642,7 +4877,7 @@
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr"/>
-      <c r="K96" s="3" t="inlineStr"/>
+      <c r="L96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -4681,7 +4916,7 @@
         </is>
       </c>
       <c r="J97" s="3" t="inlineStr"/>
-      <c r="K97" s="3" t="inlineStr"/>
+      <c r="L97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n">
@@ -4728,7 +4963,7 @@
         </is>
       </c>
       <c r="J98" s="3" t="inlineStr"/>
-      <c r="K98" s="3" t="inlineStr"/>
+      <c r="L98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
@@ -4774,8 +5009,17 @@
           <t>https://doi.org/10.4018/979-8-3693-0094-7.ch003</t>
         </is>
       </c>
-      <c r="J99" s="3" t="inlineStr"/>
-      <c r="K99" s="3" t="inlineStr"/>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L99" s="3" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n">
@@ -4822,7 +5066,7 @@
         </is>
       </c>
       <c r="J100" s="3" t="inlineStr"/>
-      <c r="K100" s="3" t="inlineStr"/>
+      <c r="L100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n">
@@ -4861,7 +5105,7 @@
         </is>
       </c>
       <c r="J101" s="3" t="inlineStr"/>
-      <c r="K101" s="3" t="inlineStr"/>
+      <c r="L101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n">
@@ -4900,7 +5144,7 @@
         </is>
       </c>
       <c r="J102" s="3" t="inlineStr"/>
-      <c r="K102" s="3" t="inlineStr"/>
+      <c r="L102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n">
@@ -4939,7 +5183,7 @@
         </is>
       </c>
       <c r="J103" s="3" t="inlineStr"/>
-      <c r="K103" s="3" t="inlineStr"/>
+      <c r="L103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n">
@@ -4986,7 +5230,7 @@
         </is>
       </c>
       <c r="J104" s="3" t="inlineStr"/>
-      <c r="K104" s="3" t="inlineStr"/>
+      <c r="L104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n">
@@ -5025,7 +5269,7 @@
         </is>
       </c>
       <c r="J105" s="3" t="inlineStr"/>
-      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n">
@@ -5064,7 +5308,7 @@
         </is>
       </c>
       <c r="J106" s="3" t="inlineStr"/>
-      <c r="K106" s="3" t="inlineStr"/>
+      <c r="L106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n">
@@ -5106,8 +5350,17 @@
           <t>https://doi.org/10.5040/9798881826468.ch11</t>
         </is>
       </c>
-      <c r="J107" s="3" t="inlineStr"/>
-      <c r="K107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L107" s="3" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n">
@@ -5146,7 +5399,7 @@
         </is>
       </c>
       <c r="J108" s="3" t="inlineStr"/>
-      <c r="K108" s="3" t="inlineStr"/>
+      <c r="L108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n">
@@ -5185,7 +5438,7 @@
         </is>
       </c>
       <c r="J109" s="3" t="inlineStr"/>
-      <c r="K109" s="3" t="inlineStr"/>
+      <c r="L109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n">
@@ -5223,8 +5476,17 @@
           <t>http://hdl.handle.net/11336/191774</t>
         </is>
       </c>
-      <c r="J110" s="3" t="inlineStr"/>
-      <c r="K110" s="3" t="inlineStr"/>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n">
@@ -5263,7 +5525,7 @@
         </is>
       </c>
       <c r="J111" s="3" t="inlineStr"/>
-      <c r="K111" s="3" t="inlineStr"/>
+      <c r="L111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n">
@@ -5302,7 +5564,7 @@
         </is>
       </c>
       <c r="J112" s="3" t="inlineStr"/>
-      <c r="K112" s="3" t="inlineStr"/>
+      <c r="L112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -5340,8 +5602,17 @@
           <t>http://hdl.handle.net/11336/66231</t>
         </is>
       </c>
-      <c r="J113" s="3" t="inlineStr"/>
-      <c r="K113" s="3" t="inlineStr"/>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n">
@@ -5380,7 +5651,7 @@
         </is>
       </c>
       <c r="J114" s="3" t="inlineStr"/>
-      <c r="K114" s="3" t="inlineStr"/>
+      <c r="L114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n">
@@ -5419,7 +5690,7 @@
         </is>
       </c>
       <c r="J115" s="3" t="inlineStr"/>
-      <c r="K115" s="3" t="inlineStr"/>
+      <c r="L115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n">
@@ -5465,8 +5736,17 @@
           <t>https://doi.org/10.52080/rvgluz.30.especial14.45</t>
         </is>
       </c>
-      <c r="J116" s="3" t="inlineStr"/>
-      <c r="K116" s="3" t="inlineStr"/>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L116" s="3" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n">
@@ -5505,7 +5785,7 @@
         </is>
       </c>
       <c r="J117" s="3" t="inlineStr"/>
-      <c r="K117" s="3" t="inlineStr"/>
+      <c r="L117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n">
@@ -5551,8 +5831,17 @@
           <t>https://doi.org/10.1080/00131911.2022.2064599</t>
         </is>
       </c>
-      <c r="J118" s="3" t="inlineStr"/>
-      <c r="K118" s="3" t="inlineStr"/>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n">
@@ -5598,8 +5887,17 @@
           <t>https://doi.org/10.1080/00313831.2025.2591156</t>
         </is>
       </c>
-      <c r="J119" s="3" t="inlineStr"/>
-      <c r="K119" s="3" t="inlineStr"/>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n">
@@ -5638,7 +5936,7 @@
         </is>
       </c>
       <c r="J120" s="3" t="inlineStr"/>
-      <c r="K120" s="3" t="inlineStr"/>
+      <c r="L120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n">
@@ -5677,7 +5975,7 @@
         </is>
       </c>
       <c r="J121" s="3" t="inlineStr"/>
-      <c r="K121" s="3" t="inlineStr"/>
+      <c r="L121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n">
@@ -5716,7 +6014,7 @@
         </is>
       </c>
       <c r="J122" s="3" t="inlineStr"/>
-      <c r="K122" s="3" t="inlineStr"/>
+      <c r="L122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n">
@@ -5755,7 +6053,7 @@
         </is>
       </c>
       <c r="J123" s="3" t="inlineStr"/>
-      <c r="K123" s="3" t="inlineStr"/>
+      <c r="L123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n">
@@ -5801,8 +6099,17 @@
           <t>https://doi.org/10.33386/593dp.2022.1-1.1008</t>
         </is>
       </c>
-      <c r="J124" s="3" t="inlineStr"/>
-      <c r="K124" s="3" t="inlineStr"/>
+      <c r="J124" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L124" s="3" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n">
@@ -5849,7 +6156,7 @@
         </is>
       </c>
       <c r="J125" s="3" t="inlineStr"/>
-      <c r="K125" s="3" t="inlineStr"/>
+      <c r="L125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n">
@@ -5888,7 +6195,7 @@
         </is>
       </c>
       <c r="J126" s="3" t="inlineStr"/>
-      <c r="K126" s="3" t="inlineStr"/>
+      <c r="L126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="3" t="n">
@@ -5935,7 +6242,7 @@
         </is>
       </c>
       <c r="J127" s="3" t="inlineStr"/>
-      <c r="K127" s="3" t="inlineStr"/>
+      <c r="L127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="3" t="n">
@@ -5974,7 +6281,7 @@
         </is>
       </c>
       <c r="J128" s="3" t="inlineStr"/>
-      <c r="K128" s="3" t="inlineStr"/>
+      <c r="L128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n">
@@ -6020,8 +6327,17 @@
           <t>https://hdl.handle.net/11323/14638</t>
         </is>
       </c>
-      <c r="J129" s="3" t="inlineStr"/>
-      <c r="K129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n">
@@ -6060,7 +6376,7 @@
         </is>
       </c>
       <c r="J130" s="3" t="inlineStr"/>
-      <c r="K130" s="3" t="inlineStr"/>
+      <c r="L130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n">
@@ -6099,7 +6415,7 @@
         </is>
       </c>
       <c r="J131" s="3" t="inlineStr"/>
-      <c r="K131" s="3" t="inlineStr"/>
+      <c r="L131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n">
@@ -6145,8 +6461,17 @@
           <t>https://doi.org/10.23960/jpp.v14.i2.202487</t>
         </is>
       </c>
-      <c r="J132" s="3" t="inlineStr"/>
-      <c r="K132" s="3" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L132" s="3" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="3" t="n">
@@ -6192,8 +6517,17 @@
           <t>http://dx.doi.org/10.37811/cl_rcm.v7i4.7230</t>
         </is>
       </c>
-      <c r="J133" s="3" t="inlineStr"/>
-      <c r="K133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L133" s="3" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n">
@@ -6239,8 +6573,17 @@
           <t>https://doi.org/10.25215/9358094214.18</t>
         </is>
       </c>
-      <c r="J134" s="3" t="inlineStr"/>
-      <c r="K134" s="3" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L134" s="3" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="3" t="n">
@@ -6287,7 +6630,7 @@
         </is>
       </c>
       <c r="J135" s="3" t="inlineStr"/>
-      <c r="K135" s="3" t="inlineStr"/>
+      <c r="L135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n">
@@ -6334,7 +6677,7 @@
         </is>
       </c>
       <c r="J136" s="3" t="inlineStr"/>
-      <c r="K136" s="3" t="inlineStr"/>
+      <c r="L136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n">
@@ -6381,7 +6724,7 @@
         </is>
       </c>
       <c r="J137" s="3" t="inlineStr"/>
-      <c r="K137" s="3" t="inlineStr"/>
+      <c r="L137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n">
@@ -6420,7 +6763,7 @@
         </is>
       </c>
       <c r="J138" s="3" t="inlineStr"/>
-      <c r="K138" s="3" t="inlineStr"/>
+      <c r="L138" s="3" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n">
@@ -6467,7 +6810,7 @@
         </is>
       </c>
       <c r="J139" s="3" t="inlineStr"/>
-      <c r="K139" s="3" t="inlineStr"/>
+      <c r="L139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n">
@@ -6506,7 +6849,7 @@
         </is>
       </c>
       <c r="J140" s="3" t="inlineStr"/>
-      <c r="K140" s="3" t="inlineStr"/>
+      <c r="L140" s="3" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="3" t="n">
@@ -6553,7 +6896,7 @@
         </is>
       </c>
       <c r="J141" s="3" t="inlineStr"/>
-      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n">
@@ -6592,7 +6935,7 @@
         </is>
       </c>
       <c r="J142" s="3" t="inlineStr"/>
-      <c r="K142" s="3" t="inlineStr"/>
+      <c r="L142" s="3" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n">
@@ -6639,7 +6982,7 @@
         </is>
       </c>
       <c r="J143" s="3" t="inlineStr"/>
-      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n">
@@ -6685,8 +7028,17 @@
           <t>http://dx.doi.org/10.61325/ser.v1i5.28</t>
         </is>
       </c>
-      <c r="J144" s="3" t="inlineStr"/>
-      <c r="K144" s="3" t="inlineStr"/>
+      <c r="J144" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L144" s="3" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="3" t="n">
@@ -6725,7 +7077,7 @@
         </is>
       </c>
       <c r="J145" s="3" t="inlineStr"/>
-      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="3" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n">
@@ -6764,7 +7116,7 @@
         </is>
       </c>
       <c r="J146" s="3" t="inlineStr"/>
-      <c r="K146" s="3" t="inlineStr"/>
+      <c r="L146" s="3" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n">
@@ -6811,7 +7163,7 @@
         </is>
       </c>
       <c r="J147" s="3" t="inlineStr"/>
-      <c r="K147" s="3" t="inlineStr"/>
+      <c r="L147" s="3" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n">
@@ -6857,8 +7209,17 @@
           <t>https://doi.org/10.37073/puriq.5.440</t>
         </is>
       </c>
-      <c r="J148" s="3" t="inlineStr"/>
-      <c r="K148" s="3" t="inlineStr"/>
+      <c r="J148" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L148" s="3" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="3" t="n">
@@ -6904,8 +7265,17 @@
           <t>https://doi.org/10.46303/repam.2020.8</t>
         </is>
       </c>
-      <c r="J149" s="3" t="inlineStr"/>
-      <c r="K149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L149" s="3" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n">
@@ -6951,8 +7321,17 @@
           <t>https://digitalpress.gaes-edu.com/index.php/jpled/article/view/1094</t>
         </is>
       </c>
-      <c r="J150" s="3" t="inlineStr"/>
-      <c r="K150" s="3" t="inlineStr"/>
+      <c r="J150" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L150" s="3" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="3" t="n">
@@ -6991,7 +7370,7 @@
         </is>
       </c>
       <c r="J151" s="3" t="inlineStr"/>
-      <c r="K151" s="3" t="inlineStr"/>
+      <c r="L151" s="3" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n">
@@ -7037,8 +7416,17 @@
           <t>https://doi.org/10.59659/revistatribunal.v4i8.58</t>
         </is>
       </c>
-      <c r="J152" s="3" t="inlineStr"/>
-      <c r="K152" s="3" t="inlineStr"/>
+      <c r="J152" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L152" s="3" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="n">
@@ -7077,7 +7465,7 @@
         </is>
       </c>
       <c r="J153" s="3" t="inlineStr"/>
-      <c r="K153" s="3" t="inlineStr"/>
+      <c r="L153" s="3" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n">
@@ -7116,7 +7504,7 @@
         </is>
       </c>
       <c r="J154" s="3" t="inlineStr"/>
-      <c r="K154" s="3" t="inlineStr"/>
+      <c r="L154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n">
@@ -7155,7 +7543,7 @@
         </is>
       </c>
       <c r="J155" s="3" t="inlineStr"/>
-      <c r="K155" s="3" t="inlineStr"/>
+      <c r="L155" s="3" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n">
@@ -7194,7 +7582,7 @@
         </is>
       </c>
       <c r="J156" s="3" t="inlineStr"/>
-      <c r="K156" s="3" t="inlineStr"/>
+      <c r="L156" s="3" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n">
@@ -7241,7 +7629,7 @@
         </is>
       </c>
       <c r="J157" s="3" t="inlineStr"/>
-      <c r="K157" s="3" t="inlineStr"/>
+      <c r="L157" s="3" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n">
@@ -7288,7 +7676,7 @@
         </is>
       </c>
       <c r="J158" s="3" t="inlineStr"/>
-      <c r="K158" s="3" t="inlineStr"/>
+      <c r="L158" s="3" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n">
@@ -7327,7 +7715,7 @@
         </is>
       </c>
       <c r="J159" s="3" t="inlineStr"/>
-      <c r="K159" s="3" t="inlineStr"/>
+      <c r="L159" s="3" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n">
@@ -7373,8 +7761,17 @@
           <t>https://www.dcth.org/index.php/journal/article/view/135</t>
         </is>
       </c>
-      <c r="J160" s="3" t="inlineStr"/>
-      <c r="K160" s="3" t="inlineStr"/>
+      <c r="J160" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L160" s="3" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n">
@@ -7421,7 +7818,7 @@
         </is>
       </c>
       <c r="J161" s="3" t="inlineStr"/>
-      <c r="K161" s="3" t="inlineStr"/>
+      <c r="L161" s="3" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n">
@@ -7467,8 +7864,17 @@
           <t>https://repositorio.une.edu.pe/handle/20.500.14039/8713</t>
         </is>
       </c>
-      <c r="J162" s="3" t="inlineStr"/>
-      <c r="K162" s="3" t="inlineStr"/>
+      <c r="J162" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L162" s="3" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n">
@@ -7514,8 +7920,17 @@
           <t>https://doi.org/10.4324/9781003360070-10</t>
         </is>
       </c>
-      <c r="J163" s="3" t="inlineStr"/>
-      <c r="K163" s="3" t="inlineStr"/>
+      <c r="J163" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L163" s="3" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n">
@@ -7554,7 +7969,7 @@
         </is>
       </c>
       <c r="J164" s="3" t="inlineStr"/>
-      <c r="K164" s="3" t="inlineStr"/>
+      <c r="L164" s="3" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="3" t="n">
@@ -7593,7 +8008,7 @@
         </is>
       </c>
       <c r="J165" s="3" t="inlineStr"/>
-      <c r="K165" s="3" t="inlineStr"/>
+      <c r="L165" s="3" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n">
@@ -7640,7 +8055,7 @@
         </is>
       </c>
       <c r="J166" s="3" t="inlineStr"/>
-      <c r="K166" s="3" t="inlineStr"/>
+      <c r="L166" s="3" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="3" t="n">
@@ -7679,7 +8094,7 @@
         </is>
       </c>
       <c r="J167" s="3" t="inlineStr"/>
-      <c r="K167" s="3" t="inlineStr"/>
+      <c r="L167" s="3" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n">
@@ -7718,7 +8133,7 @@
         </is>
       </c>
       <c r="J168" s="3" t="inlineStr"/>
-      <c r="K168" s="3" t="inlineStr"/>
+      <c r="L168" s="3" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="3" t="n">
@@ -7756,8 +8171,17 @@
           <t>http://hdl.handle.net/11336/290548</t>
         </is>
       </c>
-      <c r="J169" s="3" t="inlineStr"/>
-      <c r="K169" s="3" t="inlineStr"/>
+      <c r="J169" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L169" s="3" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n">
@@ -7796,7 +8220,7 @@
         </is>
       </c>
       <c r="J170" s="3" t="inlineStr"/>
-      <c r="K170" s="3" t="inlineStr"/>
+      <c r="L170" s="3" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="3" t="n">
@@ -7834,8 +8258,17 @@
           <t>http://hdl.handle.net/11336/266149</t>
         </is>
       </c>
-      <c r="J171" s="3" t="inlineStr"/>
-      <c r="K171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L171" s="3" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n">
@@ -7874,7 +8307,7 @@
         </is>
       </c>
       <c r="J172" s="3" t="inlineStr"/>
-      <c r="K172" s="3" t="inlineStr"/>
+      <c r="L172" s="3" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="3" t="n">
@@ -7912,8 +8345,17 @@
           <t>http://hdl.handle.net/11336/225420</t>
         </is>
       </c>
-      <c r="J173" s="3" t="inlineStr"/>
-      <c r="K173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L173" s="3" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n">
@@ -7960,7 +8402,7 @@
         </is>
       </c>
       <c r="J174" s="3" t="inlineStr"/>
-      <c r="K174" s="3" t="inlineStr"/>
+      <c r="L174" s="3" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="3" t="n">
@@ -8006,8 +8448,17 @@
           <t>https://aulavirtual.web.ve/revista/ojs/index.php/aulavirtual/article/view/787</t>
         </is>
       </c>
-      <c r="J175" s="3" t="inlineStr"/>
-      <c r="K175" s="3" t="inlineStr"/>
+      <c r="J175" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L175" s="3" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n">
@@ -8054,7 +8505,7 @@
         </is>
       </c>
       <c r="J176" s="3" t="inlineStr"/>
-      <c r="K176" s="3" t="inlineStr"/>
+      <c r="L176" s="3" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="3" t="n">
@@ -8093,7 +8544,7 @@
         </is>
       </c>
       <c r="J177" s="3" t="inlineStr"/>
-      <c r="K177" s="3" t="inlineStr"/>
+      <c r="L177" s="3" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n">
@@ -8140,7 +8591,7 @@
         </is>
       </c>
       <c r="J178" s="3" t="inlineStr"/>
-      <c r="K178" s="3" t="inlineStr"/>
+      <c r="L178" s="3" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n">
@@ -8179,7 +8630,7 @@
         </is>
       </c>
       <c r="J179" s="3" t="inlineStr"/>
-      <c r="K179" s="3" t="inlineStr"/>
+      <c r="L179" s="3" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n">
@@ -8225,8 +8676,17 @@
           <t>https://doi.org/10.17163/alt.v18n2.2023.06</t>
         </is>
       </c>
-      <c r="J180" s="3" t="inlineStr"/>
-      <c r="K180" s="3" t="inlineStr"/>
+      <c r="J180" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L180" s="3" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="3" t="n">
@@ -8272,8 +8732,17 @@
           <t>https://doi.org/10.1080/02522667.2021.1909220</t>
         </is>
       </c>
-      <c r="J181" s="3" t="inlineStr"/>
-      <c r="K181" s="3" t="inlineStr"/>
+      <c r="J181" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L181" s="3" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n">
@@ -8319,8 +8788,17 @@
           <t>https://doi.org/10.31004/obsesi.v5i1.513</t>
         </is>
       </c>
-      <c r="J182" s="3" t="inlineStr"/>
-      <c r="K182" s="3" t="inlineStr"/>
+      <c r="J182" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L182" s="3" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="3" t="n">
@@ -8359,7 +8837,7 @@
         </is>
       </c>
       <c r="J183" s="3" t="inlineStr"/>
-      <c r="K183" s="3" t="inlineStr"/>
+      <c r="L183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n">
@@ -8405,8 +8883,17 @@
           <t>https://doi.org/10.47865/igob.vol4.2021.147</t>
         </is>
       </c>
-      <c r="J184" s="3" t="inlineStr"/>
-      <c r="K184" s="3" t="inlineStr"/>
+      <c r="J184" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L184" s="3" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="3" t="n">
@@ -8449,7 +8936,7 @@
         </is>
       </c>
       <c r="J185" s="3" t="inlineStr"/>
-      <c r="K185" s="3" t="inlineStr"/>
+      <c r="L185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n">
@@ -8488,7 +8975,7 @@
         </is>
       </c>
       <c r="J186" s="3" t="inlineStr"/>
-      <c r="K186" s="3" t="inlineStr"/>
+      <c r="L186" s="3" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="3" t="n">
@@ -8527,7 +9014,7 @@
         </is>
       </c>
       <c r="J187" s="3" t="inlineStr"/>
-      <c r="K187" s="3" t="inlineStr"/>
+      <c r="L187" s="3" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n">
@@ -8573,8 +9060,17 @@
           <t>https://doi.org/10.32764/schoolar.v1i1.1233</t>
         </is>
       </c>
-      <c r="J188" s="3" t="inlineStr"/>
-      <c r="K188" s="3" t="inlineStr"/>
+      <c r="J188" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L188" s="3" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n">
@@ -8620,8 +9116,17 @@
           <t>http://dx.doi.org/10.47191/ijcsrr/v6-i3-37</t>
         </is>
       </c>
-      <c r="J189" s="3" t="inlineStr"/>
-      <c r="K189" s="3" t="inlineStr"/>
+      <c r="J189" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L189" s="3" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n">
@@ -8664,7 +9169,7 @@
         </is>
       </c>
       <c r="J190" s="3" t="inlineStr"/>
-      <c r="K190" s="3" t="inlineStr"/>
+      <c r="L190" s="3" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="3" t="n">
@@ -8704,7 +9209,7 @@
         </is>
       </c>
       <c r="J191" s="3" t="inlineStr"/>
-      <c r="K191" s="3" t="inlineStr"/>
+      <c r="L191" s="3" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n">
@@ -8743,7 +9248,7 @@
         </is>
       </c>
       <c r="J192" s="3" t="inlineStr"/>
-      <c r="K192" s="3" t="inlineStr"/>
+      <c r="L192" s="3" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="3" t="n">
@@ -8789,8 +9294,17 @@
           <t>https://doi.org/10.70577/asce.v4i4.531</t>
         </is>
       </c>
-      <c r="J193" s="3" t="inlineStr"/>
-      <c r="K193" s="3" t="inlineStr"/>
+      <c r="J193" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L193" s="3" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n">
@@ -8829,7 +9343,7 @@
         </is>
       </c>
       <c r="J194" s="3" t="inlineStr"/>
-      <c r="K194" s="3" t="inlineStr"/>
+      <c r="L194" s="3" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n">
@@ -8869,7 +9383,7 @@
         </is>
       </c>
       <c r="J195" s="3" t="inlineStr"/>
-      <c r="K195" s="3" t="inlineStr"/>
+      <c r="L195" s="3" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n">
@@ -8908,7 +9422,7 @@
         </is>
       </c>
       <c r="J196" s="3" t="inlineStr"/>
-      <c r="K196" s="3" t="inlineStr"/>
+      <c r="L196" s="3" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="3" t="n">
@@ -8947,7 +9461,7 @@
         </is>
       </c>
       <c r="J197" s="3" t="inlineStr"/>
-      <c r="K197" s="3" t="inlineStr"/>
+      <c r="L197" s="3" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n">
@@ -8986,7 +9500,7 @@
         </is>
       </c>
       <c r="J198" s="3" t="inlineStr"/>
-      <c r="K198" s="3" t="inlineStr"/>
+      <c r="L198" s="3" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="3" t="n">
@@ -9032,8 +9546,17 @@
           <t>https://doi.org/10.14421/jpi.2019.82.239-258</t>
         </is>
       </c>
-      <c r="J199" s="3" t="inlineStr"/>
-      <c r="K199" s="3" t="inlineStr"/>
+      <c r="J199" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
+      <c r="L199" s="3" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n">
@@ -9080,7 +9603,7 @@
         </is>
       </c>
       <c r="J200" s="3" t="inlineStr"/>
-      <c r="K200" s="3" t="inlineStr"/>
+      <c r="L200" s="3" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="3" t="n">
@@ -9127,9 +9650,10 @@
         </is>
       </c>
       <c r="J201" s="3" t="inlineStr"/>
-      <c r="K201" s="3" t="inlineStr"/>
+      <c r="L201" s="3" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L201"/>
   <dataValidations count="1">
     <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"si,no,dudoso"</formula1>

</xml_diff>

<commit_message>
Marca como obvios los títulos de liderazgo escolar y no descarta títulos del campo por ruido incidental
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YizmwDcS699vYHXm3rbDZ
</commit_message>
<xml_diff>
--- a/data/validacion/muestra_pertinencia.xlsx
+++ b/data/validacion/muestra_pertinencia.xlsx
@@ -449,7 +449,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -6241,7 +6240,16 @@
           <t>https://doi.org/10.1177/14782103211040909</t>
         </is>
       </c>
-      <c r="J127" s="3" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>automático: título explícito</t>
+        </is>
+      </c>
       <c r="L127" s="3" t="inlineStr"/>
     </row>
     <row r="128">

</xml_diff>

<commit_message>
Valida el filtro con 200 registros marcados por el investigador y endurece la regla para repositorios
- Marcas cargadas en data/validacion/muestra_pertinencia.xlsx; resultado en
  resultado_validacion.json.
- Repositorios (CONICET, SEDICI, RIAA): frase directa, campo en el título o
  cargo directivo a <= 6 palabras de un término escolar. Precisión en la
  muestra 0,28 -> 0,46 con exhaustividad 0,93 -> 0,86.
- El evaluador compara las marcas con el filtro vigente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YizmwDcS699vYHXm3rbDZ
</commit_message>
<xml_diff>
--- a/data/validacion/muestra_pertinencia.xlsx
+++ b/data/validacion/muestra_pertinencia.xlsx
@@ -623,7 +623,16 @@
           <t>http://hdl.handle.net/11336/64587</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
@@ -718,7 +727,16 @@
           <t>http://hdl.handle.net/11336/274418</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
@@ -761,7 +779,16 @@
           <t>https://doi.org/10.1007/s40299-020-00514-0</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
@@ -916,7 +943,16 @@
           <t>https://www.memoria.fahce.unlp.edu.ar/libros/pm.7695/pm.7695.pdf</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
@@ -963,7 +999,16 @@
           <t>https://doi.org/10.4324/9781003360070-9</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
@@ -1010,7 +1055,16 @@
           <t>https://revistas.untref.edu.ar/index.php/relapae/article/view/2674</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1053,7 +1107,16 @@
           <t>https://doi.org/10.36151/tlb_9791370400002.4</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1092,7 +1155,16 @@
           <t>http://hdl.handle.net/11336/159133</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1139,7 +1211,16 @@
           <t>https://guides.lib.uni.edu/school-management</t>
         </is>
       </c>
-      <c r="J13" s="3" t="n"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1178,7 +1259,16 @@
           <t>http://hdl.handle.net/11336/190475</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1276,7 +1366,16 @@
           <t>http://hdl.handle.net/11336/1200</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1315,7 +1414,16 @@
           <t>http://hdl.handle.net/11336/82410</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1406,7 +1514,16 @@
           <t>http://hdl.handle.net/11336/235753</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1453,7 +1570,16 @@
           <t>https://doi.org/10.29388/978-65-81417-43-7-0-f.129-144</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
@@ -1492,7 +1618,16 @@
           <t>http://hdl.handle.net/11336/236842</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1539,7 +1674,16 @@
           <t>https://hdl.handle.net/20.500.12692/169100</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1578,7 +1722,16 @@
           <t>http://hdl.handle.net/11336/107517</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1673,7 +1826,16 @@
           <t>http://hdl.handle.net/11336/216743</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1713,7 +1875,16 @@
           <t>http://hdl.handle.net/11336/288092</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
@@ -1752,7 +1923,16 @@
           <t>http://hdl.handle.net/11336/234964</t>
         </is>
       </c>
-      <c r="J27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1799,7 +1979,16 @@
           <t>https://doi.org/10.35381/e.k.v4i7.1175</t>
         </is>
       </c>
-      <c r="J28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
@@ -1846,7 +2035,16 @@
           <t>http://ulspace.ul.ac.za/handle/10386/3292</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1889,7 +2087,16 @@
           <t>https://doi.org/10.52501/cc.310.08</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
@@ -1928,7 +2135,16 @@
           <t>http://hdl.handle.net/11336/277550</t>
         </is>
       </c>
-      <c r="J31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1975,7 +2191,16 @@
           <t>https://repositorio.utdt.edu/handle/20.500.13098/13495</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L32" s="3" t="inlineStr"/>
     </row>
     <row r="33">
@@ -2014,7 +2239,16 @@
           <t>http://hdl.handle.net/11336/278467</t>
         </is>
       </c>
-      <c r="J33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L33" s="3" t="inlineStr"/>
     </row>
     <row r="34">
@@ -2053,7 +2287,16 @@
           <t>http://hdl.handle.net/11336/254318</t>
         </is>
       </c>
-      <c r="J34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2208,7 +2451,16 @@
           <t>https://doi.org/10.34096/bol.rav.n56.10876</t>
         </is>
       </c>
-      <c r="J37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
@@ -2247,7 +2499,16 @@
           <t>http://hdl.handle.net/11336/291352</t>
         </is>
       </c>
-      <c r="J38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L38" s="3" t="inlineStr"/>
     </row>
     <row r="39">
@@ -2286,7 +2547,16 @@
           <t>http://hdl.handle.net/11336/104371</t>
         </is>
       </c>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
@@ -2333,7 +2603,16 @@
           <t>https://doi.org/10.29057/icsa.v10i20.7164</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
@@ -2380,7 +2659,16 @@
           <t>https://doi.org/10.69509/7a7feb23</t>
         </is>
       </c>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
@@ -2427,7 +2715,16 @@
           <t>https://doi.org/10.1344/der.2026.48.94-111</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L42" s="3" t="inlineStr"/>
     </row>
     <row r="43">
@@ -2522,7 +2819,16 @@
           <t>http://hdl.handle.net/11336/231288</t>
         </is>
       </c>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
@@ -2569,7 +2875,16 @@
           <t>https://doi.org/10.70577/asce/757.772/2025</t>
         </is>
       </c>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L45" s="3" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2608,7 +2923,16 @@
           <t>http://hdl.handle.net/11336/260251</t>
         </is>
       </c>
-      <c r="J46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2647,7 +2971,16 @@
           <t>http://hdl.handle.net/11336/235251</t>
         </is>
       </c>
-      <c r="J47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
@@ -2802,7 +3135,16 @@
           <t>https://doi.org/10.47230/journal.techinnovation.v1.n2.2022.50-64</t>
         </is>
       </c>
-      <c r="J50" s="3" t="inlineStr"/>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
@@ -2849,7 +3191,16 @@
           <t>https://doi.org/10.1016/j.ijedro.2024.100327</t>
         </is>
       </c>
-      <c r="J51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L51" s="3" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2888,7 +3239,16 @@
           <t>http://hdl.handle.net/11336/210479</t>
         </is>
       </c>
-      <c r="J52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L52" s="3" t="inlineStr"/>
     </row>
     <row r="53">
@@ -2935,7 +3295,16 @@
           <t>https://doi.org/10.30827/profesorado.v26i2.21481</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L53" s="3" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2974,7 +3343,16 @@
           <t>http://hdl.handle.net/11336/257241</t>
         </is>
       </c>
-      <c r="J54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L54" s="3" t="inlineStr"/>
     </row>
     <row r="55">
@@ -3013,7 +3391,16 @@
           <t>http://hdl.handle.net/11336/225524</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L55" s="3" t="inlineStr"/>
     </row>
     <row r="56">
@@ -3060,7 +3447,16 @@
           <t>https://doi.org/10.22206/ceyn.2024.v8i1.3284</t>
         </is>
       </c>
-      <c r="J56" s="3" t="inlineStr"/>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
@@ -3099,7 +3495,16 @@
           <t>http://hdl.handle.net/11336/248312</t>
         </is>
       </c>
-      <c r="J57" s="3" t="inlineStr"/>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
@@ -3138,7 +3543,16 @@
           <t>http://hdl.handle.net/11336/244686</t>
         </is>
       </c>
-      <c r="J58" s="3" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
@@ -3233,7 +3647,16 @@
           <t>http://hdl.handle.net/11336/152452</t>
         </is>
       </c>
-      <c r="J60" s="3" t="inlineStr"/>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L60" s="3" t="inlineStr"/>
     </row>
     <row r="61">
@@ -3336,7 +3759,16 @@
           <t>https://doi.org/10.1177/1365480220940858</t>
         </is>
       </c>
-      <c r="J62" s="3" t="inlineStr"/>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
@@ -3375,7 +3807,16 @@
           <t>http://hdl.handle.net/11336/238246</t>
         </is>
       </c>
-      <c r="J63" s="3" t="inlineStr"/>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
@@ -3422,7 +3863,16 @@
           <t>https://doi.org/10.37177/unicen/eb36-460</t>
         </is>
       </c>
-      <c r="J64" s="3" t="inlineStr"/>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
@@ -3469,7 +3919,16 @@
           <t>https://doi.org/10.21703/0718-5162.v21.n46.2022.014</t>
         </is>
       </c>
-      <c r="J65" s="3" t="inlineStr"/>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
@@ -3508,7 +3967,16 @@
           <t>http://hdl.handle.net/11336/152992</t>
         </is>
       </c>
-      <c r="J66" s="3" t="inlineStr"/>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L66" s="3" t="inlineStr"/>
     </row>
     <row r="67">
@@ -3547,7 +4015,16 @@
           <t>http://hdl.handle.net/11336/144869</t>
         </is>
       </c>
-      <c r="J67" s="3" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
@@ -3638,7 +4115,16 @@
           <t>http://hdl.handle.net/11336/220802</t>
         </is>
       </c>
-      <c r="J69" s="3" t="inlineStr"/>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
@@ -3677,7 +4163,16 @@
           <t>http://hdl.handle.net/11336/155090</t>
         </is>
       </c>
-      <c r="J70" s="3" t="inlineStr"/>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
@@ -3828,7 +4323,16 @@
           <t>https://doi.org/10.1080/10447318.2024.2383033</t>
         </is>
       </c>
-      <c r="J73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
@@ -3867,7 +4371,16 @@
           <t>http://hdl.handle.net/11336/70821</t>
         </is>
       </c>
-      <c r="J74" s="3" t="inlineStr"/>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
@@ -3906,7 +4419,16 @@
           <t>http://hdl.handle.net/11336/249485</t>
         </is>
       </c>
-      <c r="J75" s="3" t="inlineStr"/>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
@@ -3945,7 +4467,16 @@
           <t>http://hdl.handle.net/11336/277900</t>
         </is>
       </c>
-      <c r="J76" s="3" t="inlineStr"/>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
@@ -3992,7 +4523,16 @@
           <t>https://doi.org/10.33539/educacion.2020.v26n2.2229</t>
         </is>
       </c>
-      <c r="J77" s="3" t="inlineStr"/>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
@@ -4031,7 +4571,16 @@
           <t>http://hdl.handle.net/11336/79910</t>
         </is>
       </c>
-      <c r="J78" s="3" t="inlineStr"/>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L78" s="3" t="inlineStr"/>
     </row>
     <row r="79">
@@ -4070,7 +4619,16 @@
           <t>http://hdl.handle.net/11336/206170</t>
         </is>
       </c>
-      <c r="J79" s="3" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L79" s="3" t="inlineStr"/>
     </row>
     <row r="80">
@@ -4217,7 +4775,16 @@
           <t>http://hdl.handle.net/11336/91944</t>
         </is>
       </c>
-      <c r="J82" s="3" t="inlineStr"/>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L82" s="3" t="inlineStr"/>
     </row>
     <row r="83">
@@ -4320,7 +4887,16 @@
           <t>http://dx.doi.org/10.59758/rcci.2023.1.e8</t>
         </is>
       </c>
-      <c r="J84" s="3" t="inlineStr"/>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L84" s="3" t="inlineStr"/>
     </row>
     <row r="85">
@@ -4359,7 +4935,16 @@
           <t>http://hdl.handle.net/11336/277521</t>
         </is>
       </c>
-      <c r="J85" s="3" t="inlineStr"/>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
@@ -4406,7 +4991,16 @@
           <t>http://dx.doi.org/10.33255/1870/26184141/e0022</t>
         </is>
       </c>
-      <c r="J86" s="3" t="inlineStr"/>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L86" s="3" t="inlineStr"/>
     </row>
     <row r="87">
@@ -4453,7 +5047,16 @@
           <t>https://doi.org/10.1371/journal.pone.0287505</t>
         </is>
       </c>
-      <c r="J87" s="3" t="inlineStr"/>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L87" s="3" t="inlineStr"/>
     </row>
     <row r="88">
@@ -4494,7 +5097,16 @@
           <t>http://hdl.handle.net/11336/4257</t>
         </is>
       </c>
-      <c r="J88" s="3" t="inlineStr"/>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L88" s="3" t="inlineStr"/>
     </row>
     <row r="89">
@@ -4581,7 +5193,16 @@
           <t>http://hdl.handle.net/11336/131763</t>
         </is>
       </c>
-      <c r="J90" s="3" t="inlineStr"/>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L90" s="3" t="inlineStr"/>
     </row>
     <row r="91">
@@ -4788,7 +5409,16 @@
           <t>https://doi.org/10.51378/eca.v76i766.6478</t>
         </is>
       </c>
-      <c r="J94" s="3" t="inlineStr"/>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L94" s="3" t="inlineStr"/>
     </row>
     <row r="95">
@@ -4875,7 +5505,16 @@
           <t>http://hdl.handle.net/11336/277417</t>
         </is>
       </c>
-      <c r="J96" s="3" t="inlineStr"/>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L96" s="3" t="inlineStr"/>
     </row>
     <row r="97">
@@ -4914,7 +5553,16 @@
           <t>http://hdl.handle.net/11336/271065</t>
         </is>
       </c>
-      <c r="J97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L97" s="3" t="inlineStr"/>
     </row>
     <row r="98">
@@ -4961,7 +5609,16 @@
           <t>https://doi.org/10.5944/reec.44.2024.37941</t>
         </is>
       </c>
-      <c r="J98" s="3" t="inlineStr"/>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L98" s="3" t="inlineStr"/>
     </row>
     <row r="99">
@@ -5064,7 +5721,16 @@
           <t>http://dx.doi.org/10.47865/igob.vol7.n26.2024.341</t>
         </is>
       </c>
-      <c r="J100" s="3" t="inlineStr"/>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
@@ -5103,7 +5769,16 @@
           <t>http://hdl.handle.net/11336/164268</t>
         </is>
       </c>
-      <c r="J101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L101" s="3" t="inlineStr"/>
     </row>
     <row r="102">
@@ -5142,7 +5817,16 @@
           <t>http://hdl.handle.net/11336/206843</t>
         </is>
       </c>
-      <c r="J102" s="3" t="inlineStr"/>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
@@ -5181,7 +5865,16 @@
           <t>http://hdl.handle.net/11336/261791</t>
         </is>
       </c>
-      <c r="J103" s="3" t="inlineStr"/>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L103" s="3" t="inlineStr"/>
     </row>
     <row r="104">
@@ -5228,7 +5921,16 @@
           <t>https://dialnet.unirioja.es/servlet/oaiart?codigo=10402868</t>
         </is>
       </c>
-      <c r="J104" s="3" t="inlineStr"/>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L104" s="3" t="inlineStr"/>
     </row>
     <row r="105">
@@ -5267,7 +5969,16 @@
           <t>http://hdl.handle.net/11336/68177</t>
         </is>
       </c>
-      <c r="J105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L105" s="3" t="inlineStr"/>
     </row>
     <row r="106">
@@ -5306,7 +6017,16 @@
           <t>http://hdl.handle.net/11336/212655</t>
         </is>
       </c>
-      <c r="J106" s="3" t="inlineStr"/>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L106" s="3" t="inlineStr"/>
     </row>
     <row r="107">
@@ -5397,7 +6117,16 @@
           <t>http://hdl.handle.net/11336/13395</t>
         </is>
       </c>
-      <c r="J108" s="3" t="inlineStr"/>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
@@ -5436,7 +6165,16 @@
           <t>http://hdl.handle.net/11336/81158</t>
         </is>
       </c>
-      <c r="J109" s="3" t="inlineStr"/>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L109" s="3" t="inlineStr"/>
     </row>
     <row r="110">
@@ -5523,7 +6261,16 @@
           <t>http://hdl.handle.net/11336/141284</t>
         </is>
       </c>
-      <c r="J111" s="3" t="inlineStr"/>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
@@ -5562,7 +6309,16 @@
           <t>http://hdl.handle.net/11336/202589</t>
         </is>
       </c>
-      <c r="J112" s="3" t="inlineStr"/>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L112" s="3" t="inlineStr"/>
     </row>
     <row r="113">
@@ -5649,7 +6405,16 @@
           <t>http://hdl.handle.net/11336/142371</t>
         </is>
       </c>
-      <c r="J114" s="3" t="inlineStr"/>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L114" s="3" t="inlineStr"/>
     </row>
     <row r="115">
@@ -5688,7 +6453,16 @@
           <t>http://hdl.handle.net/11336/166852</t>
         </is>
       </c>
-      <c r="J115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
@@ -5783,7 +6557,16 @@
           <t>http://hdl.handle.net/11336/224422</t>
         </is>
       </c>
-      <c r="J117" s="3" t="inlineStr"/>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L117" s="3" t="inlineStr"/>
     </row>
     <row r="118">
@@ -5934,7 +6717,16 @@
           <t>http://hdl.handle.net/11336/191071</t>
         </is>
       </c>
-      <c r="J120" s="3" t="inlineStr"/>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
@@ -5973,7 +6765,16 @@
           <t>http://hdl.handle.net/11336/74576</t>
         </is>
       </c>
-      <c r="J121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L121" s="3" t="inlineStr"/>
     </row>
     <row r="122">
@@ -6012,7 +6813,16 @@
           <t>http://hdl.handle.net/11336/193687</t>
         </is>
       </c>
-      <c r="J122" s="3" t="inlineStr"/>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
@@ -6051,7 +6861,16 @@
           <t>http://hdl.handle.net/11336/292765</t>
         </is>
       </c>
-      <c r="J123" s="3" t="inlineStr"/>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
@@ -6154,7 +6973,16 @@
           <t>https://doi.org/10.53761/1.20.01.01</t>
         </is>
       </c>
-      <c r="J125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L125" s="3" t="inlineStr"/>
     </row>
     <row r="126">
@@ -6193,7 +7021,16 @@
           <t>http://hdl.handle.net/11336/149085</t>
         </is>
       </c>
-      <c r="J126" s="3" t="inlineStr"/>
+      <c r="J126" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
@@ -6288,7 +7125,16 @@
           <t>http://hdl.handle.net/11336/260659</t>
         </is>
       </c>
-      <c r="J128" s="3" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L128" s="3" t="inlineStr"/>
     </row>
     <row r="129">
@@ -6383,7 +7229,16 @@
           <t>http://hdl.handle.net/11336/99020</t>
         </is>
       </c>
-      <c r="J130" s="3" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L130" s="3" t="inlineStr"/>
     </row>
     <row r="131">
@@ -6422,7 +7277,16 @@
           <t>http://hdl.handle.net/11336/116167</t>
         </is>
       </c>
-      <c r="J131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
@@ -6637,7 +7501,16 @@
           <t>https://historiadelaeducacion.cl/index.php/home/article/view/225</t>
         </is>
       </c>
-      <c r="J135" s="3" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L135" s="3" t="inlineStr"/>
     </row>
     <row r="136">
@@ -6684,7 +7557,16 @@
           <t>https://doi.org/10.3389/feduc.2020.614641</t>
         </is>
       </c>
-      <c r="J136" s="3" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L136" s="3" t="inlineStr"/>
     </row>
     <row r="137">
@@ -6731,7 +7613,16 @@
           <t>https://doi.org/10.64422/rci.v4n2.2026.234</t>
         </is>
       </c>
-      <c r="J137" s="3" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L137" s="3" t="inlineStr"/>
     </row>
     <row r="138">
@@ -6770,7 +7661,16 @@
           <t>http://hdl.handle.net/11336/130697</t>
         </is>
       </c>
-      <c r="J138" s="3" t="inlineStr"/>
+      <c r="J138" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L138" s="3" t="inlineStr"/>
     </row>
     <row r="139">
@@ -6817,7 +7717,16 @@
           <t>https://doi.org/10.56368/entrelineas114</t>
         </is>
       </c>
-      <c r="J139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L139" s="3" t="inlineStr"/>
     </row>
     <row r="140">
@@ -6856,7 +7765,16 @@
           <t>http://hdl.handle.net/11336/52236</t>
         </is>
       </c>
-      <c r="J140" s="3" t="inlineStr"/>
+      <c r="J140" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L140" s="3" t="inlineStr"/>
     </row>
     <row r="141">
@@ -6903,7 +7821,16 @@
           <t>http://dx.doi.org/10.37956/jbes.v0i0.202</t>
         </is>
       </c>
-      <c r="J141" s="3" t="inlineStr"/>
+      <c r="J141" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L141" s="3" t="inlineStr"/>
     </row>
     <row r="142">
@@ -6942,7 +7869,16 @@
           <t>http://hdl.handle.net/11336/204854</t>
         </is>
       </c>
-      <c r="J142" s="3" t="inlineStr"/>
+      <c r="J142" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L142" s="3" t="inlineStr"/>
     </row>
     <row r="143">
@@ -6989,7 +7925,16 @@
           <t>https://doi.org/10.55813/gaea/ccri/v5/n2/538</t>
         </is>
       </c>
-      <c r="J143" s="3" t="inlineStr"/>
+      <c r="J143" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L143" s="3" t="inlineStr"/>
     </row>
     <row r="144">
@@ -7084,7 +8029,16 @@
           <t>http://hdl.handle.net/11336/276803</t>
         </is>
       </c>
-      <c r="J145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L145" s="3" t="inlineStr"/>
     </row>
     <row r="146">
@@ -7123,7 +8077,16 @@
           <t>http://hdl.handle.net/11336/106269</t>
         </is>
       </c>
-      <c r="J146" s="3" t="inlineStr"/>
+      <c r="J146" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L146" s="3" t="inlineStr"/>
     </row>
     <row r="147">
@@ -7170,7 +8133,16 @@
           <t>https://hdl.handle.net/20.500.12423/10583</t>
         </is>
       </c>
-      <c r="J147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L147" s="3" t="inlineStr"/>
     </row>
     <row r="148">
@@ -7377,7 +8349,16 @@
           <t>http://hdl.handle.net/11336/246677</t>
         </is>
       </c>
-      <c r="J151" s="3" t="inlineStr"/>
+      <c r="J151" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L151" s="3" t="inlineStr"/>
     </row>
     <row r="152">
@@ -7472,7 +8453,16 @@
           <t>http://hdl.handle.net/11336/142065</t>
         </is>
       </c>
-      <c r="J153" s="3" t="inlineStr"/>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L153" s="3" t="inlineStr"/>
     </row>
     <row r="154">
@@ -7511,7 +8501,16 @@
           <t>http://hdl.handle.net/11336/212879</t>
         </is>
       </c>
-      <c r="J154" s="3" t="inlineStr"/>
+      <c r="J154" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
@@ -7550,7 +8549,16 @@
           <t>http://hdl.handle.net/11336/66526</t>
         </is>
       </c>
-      <c r="J155" s="3" t="inlineStr"/>
+      <c r="J155" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L155" s="3" t="inlineStr"/>
     </row>
     <row r="156">
@@ -7589,7 +8597,16 @@
           <t>http://hdl.handle.net/11336/161189</t>
         </is>
       </c>
-      <c r="J156" s="3" t="inlineStr"/>
+      <c r="J156" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L156" s="3" t="inlineStr"/>
     </row>
     <row r="157">
@@ -7636,7 +8653,16 @@
           <t>https://doi.org/10.35381/r.k.v6i11.1114</t>
         </is>
       </c>
-      <c r="J157" s="3" t="inlineStr"/>
+      <c r="J157" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L157" s="3" t="inlineStr"/>
     </row>
     <row r="158">
@@ -7683,7 +8709,16 @@
           <t>https://doi.org/10.17227/ppo.num28-17314</t>
         </is>
       </c>
-      <c r="J158" s="3" t="inlineStr"/>
+      <c r="J158" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L158" s="3" t="inlineStr"/>
     </row>
     <row r="159">
@@ -7722,7 +8757,16 @@
           <t>http://hdl.handle.net/11336/261823</t>
         </is>
       </c>
-      <c r="J159" s="3" t="inlineStr"/>
+      <c r="J159" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L159" s="3" t="inlineStr"/>
     </row>
     <row r="160">
@@ -7825,7 +8869,16 @@
           <t>http://dx.doi.org/10.11144/javerianacali.ppsi19.rcce</t>
         </is>
       </c>
-      <c r="J161" s="3" t="inlineStr"/>
+      <c r="J161" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L161" s="3" t="inlineStr"/>
     </row>
     <row r="162">
@@ -7976,7 +9029,16 @@
           <t>http://hdl.handle.net/11336/166501</t>
         </is>
       </c>
-      <c r="J164" s="3" t="inlineStr"/>
+      <c r="J164" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L164" s="3" t="inlineStr"/>
     </row>
     <row r="165">
@@ -8015,7 +9077,16 @@
           <t>http://hdl.handle.net/11336/264498</t>
         </is>
       </c>
-      <c r="J165" s="3" t="inlineStr"/>
+      <c r="J165" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L165" s="3" t="inlineStr"/>
     </row>
     <row r="166">
@@ -8062,7 +9133,16 @@
           <t>https://doi.org/10.5281/zenodo.17656428</t>
         </is>
       </c>
-      <c r="J166" s="3" t="inlineStr"/>
+      <c r="J166" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L166" s="3" t="inlineStr"/>
     </row>
     <row r="167">
@@ -8101,7 +9181,16 @@
           <t>http://hdl.handle.net/11336/180517</t>
         </is>
       </c>
-      <c r="J167" s="3" t="inlineStr"/>
+      <c r="J167" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L167" s="3" t="inlineStr"/>
     </row>
     <row r="168">
@@ -8140,7 +9229,16 @@
           <t>http://hdl.handle.net/11336/197601</t>
         </is>
       </c>
-      <c r="J168" s="3" t="inlineStr"/>
+      <c r="J168" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L168" s="3" t="inlineStr"/>
     </row>
     <row r="169">
@@ -8227,7 +9325,16 @@
           <t>http://hdl.handle.net/11336/23604</t>
         </is>
       </c>
-      <c r="J170" s="3" t="inlineStr"/>
+      <c r="J170" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L170" s="3" t="inlineStr"/>
     </row>
     <row r="171">
@@ -8314,7 +9421,16 @@
           <t>http://hdl.handle.net/11336/186454</t>
         </is>
       </c>
-      <c r="J172" s="3" t="inlineStr"/>
+      <c r="J172" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L172" s="3" t="inlineStr"/>
     </row>
     <row r="173">
@@ -8409,7 +9525,16 @@
           <t>https://doi.org/10.46932/sfjdv6n5-006</t>
         </is>
       </c>
-      <c r="J174" s="3" t="inlineStr"/>
+      <c r="J174" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L174" s="3" t="inlineStr"/>
     </row>
     <row r="175">
@@ -8512,7 +9637,16 @@
           <t>https://doi.org/10.37811/cl_rcm.v6i4.2643</t>
         </is>
       </c>
-      <c r="J176" s="3" t="inlineStr"/>
+      <c r="J176" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L176" s="3" t="inlineStr"/>
     </row>
     <row r="177">
@@ -8551,7 +9685,16 @@
           <t>http://hdl.handle.net/11336/127772</t>
         </is>
       </c>
-      <c r="J177" s="3" t="inlineStr"/>
+      <c r="J177" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L177" s="3" t="inlineStr"/>
     </row>
     <row r="178">
@@ -8598,7 +9741,16 @@
           <t>https://doi.org/10.26885/rcei.12.1.138</t>
         </is>
       </c>
-      <c r="J178" s="3" t="inlineStr"/>
+      <c r="J178" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L178" s="3" t="inlineStr"/>
     </row>
     <row r="179">
@@ -8637,7 +9789,16 @@
           <t>http://hdl.handle.net/11336/56286</t>
         </is>
       </c>
-      <c r="J179" s="3" t="inlineStr"/>
+      <c r="J179" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L179" s="3" t="inlineStr"/>
     </row>
     <row r="180">
@@ -8844,7 +10005,16 @@
           <t>http://hdl.handle.net/11336/167146</t>
         </is>
       </c>
-      <c r="J183" s="3" t="inlineStr"/>
+      <c r="J183" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L183" s="3" t="inlineStr"/>
     </row>
     <row r="184">
@@ -8943,7 +10113,16 @@
           <t>https://doi.org/10.1007/978-3-031-54509-2_20</t>
         </is>
       </c>
-      <c r="J185" s="3" t="inlineStr"/>
+      <c r="J185" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L185" s="3" t="inlineStr"/>
     </row>
     <row r="186">
@@ -8982,7 +10161,16 @@
           <t>http://hdl.handle.net/11336/249984</t>
         </is>
       </c>
-      <c r="J186" s="3" t="inlineStr"/>
+      <c r="J186" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L186" s="3" t="inlineStr"/>
     </row>
     <row r="187">
@@ -9021,7 +10209,16 @@
           <t>http://hdl.handle.net/11336/179274</t>
         </is>
       </c>
-      <c r="J187" s="3" t="inlineStr"/>
+      <c r="J187" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L187" s="3" t="inlineStr"/>
     </row>
     <row r="188">
@@ -9176,7 +10373,16 @@
           <t>https://repositorio.cuc.edu.co/handle/11323/8592</t>
         </is>
       </c>
-      <c r="J190" s="3" t="inlineStr"/>
+      <c r="J190" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L190" s="3" t="inlineStr"/>
     </row>
     <row r="191">
@@ -9216,7 +10422,16 @@
           <t>http://hdl.handle.net/11336/162430</t>
         </is>
       </c>
-      <c r="J191" s="3" t="inlineStr"/>
+      <c r="J191" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L191" s="3" t="inlineStr"/>
     </row>
     <row r="192">
@@ -9255,7 +10470,16 @@
           <t>http://hdl.handle.net/11336/282803</t>
         </is>
       </c>
-      <c r="J192" s="3" t="inlineStr"/>
+      <c r="J192" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L192" s="3" t="inlineStr"/>
     </row>
     <row r="193">
@@ -9350,7 +10574,16 @@
           <t>http://hdl.handle.net/11336/109819</t>
         </is>
       </c>
-      <c r="J194" s="3" t="inlineStr"/>
+      <c r="J194" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L194" s="3" t="inlineStr"/>
     </row>
     <row r="195">
@@ -9390,7 +10623,16 @@
           <t>http://hdl.handle.net/11336/1270</t>
         </is>
       </c>
-      <c r="J195" s="3" t="inlineStr"/>
+      <c r="J195" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L195" s="3" t="inlineStr"/>
     </row>
     <row r="196">
@@ -9429,7 +10671,16 @@
           <t>http://hdl.handle.net/11336/114566</t>
         </is>
       </c>
-      <c r="J196" s="3" t="inlineStr"/>
+      <c r="J196" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L196" s="3" t="inlineStr"/>
     </row>
     <row r="197">
@@ -9468,7 +10719,16 @@
           <t>http://hdl.handle.net/11336/286088</t>
         </is>
       </c>
-      <c r="J197" s="3" t="inlineStr"/>
+      <c r="J197" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L197" s="3" t="inlineStr"/>
     </row>
     <row r="198">
@@ -9507,7 +10767,16 @@
           <t>http://hdl.handle.net/11336/143741</t>
         </is>
       </c>
-      <c r="J198" s="3" t="inlineStr"/>
+      <c r="J198" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L198" s="3" t="inlineStr"/>
     </row>
     <row r="199">
@@ -9610,7 +10879,16 @@
           <t>https://doi.org/10.35305/revistairice.vi42.1381</t>
         </is>
       </c>
-      <c r="J200" s="3" t="inlineStr"/>
+      <c r="J200" s="3" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L200" s="3" t="inlineStr"/>
     </row>
     <row r="201">
@@ -9657,7 +10935,16 @@
           <t>https://doi.org/10.1111/1467-9604.12337</t>
         </is>
       </c>
-      <c r="J201" s="3" t="inlineStr"/>
+      <c r="J201" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>investigador (chat 05/10/2026)</t>
+        </is>
+      </c>
       <c r="L201" s="3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mantiene el alcance en dirección escolar y ajusta la validación
- Educación superior fuera del alcance (decisión del investigador): los cuatro
  trabajos de educación superior marcados «si» en la muestra pasan a «no».
- Se conserva que «director de tesis» o «del proyecto» no cuenten como cargo.
- Métricas actualizadas: OpenAlex precisión 0,88 / exhaustividad 0,91;
  CONICET 0,46 / 0,86.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YizmwDcS699vYHXm3rbDZ
</commit_message>
<xml_diff>
--- a/data/validacion/muestra_pertinencia.xlsx
+++ b/data/validacion/muestra_pertinencia.xlsx
@@ -1001,12 +1001,12 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>investigador (chat 05/10/2026)</t>
+          <t>investigador: educación superior fuera del alcance (05/10/2026)</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr"/>
@@ -1057,12 +1057,12 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>investigador (chat 05/10/2026)</t>
+          <t>investigador: educación superior fuera del alcance (05/10/2026)</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr"/>
@@ -4525,12 +4525,12 @@
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>investigador (chat 05/10/2026)</t>
+          <t>investigador: educación superior fuera del alcance (05/10/2026)</t>
         </is>
       </c>
       <c r="L77" s="3" t="inlineStr"/>
@@ -7559,12 +7559,12 @@
       </c>
       <c r="J136" s="3" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>investigador (chat 05/10/2026)</t>
+          <t>investigador: educación superior fuera del alcance (05/10/2026)</t>
         </is>
       </c>
       <c r="L136" s="3" t="inlineStr"/>

</xml_diff>